<commit_message>
feat: guardado incremental + quitar mención de Facebook/Instagram del formulario para vendedores
</commit_message>
<xml_diff>
--- a/public/demos/enlaceintegral/top-clientes/plantilla-top20.xlsx
+++ b/public/demos/enlaceintegral/top-clientes/plantilla-top20.xlsx
@@ -554,7 +554,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Vamos a construir una base de datos con tus 20 mejores clientes (los más leales, los que más te compran, los que renuevan sin problema). Con esta información, Enlace Integral podrá anunciarse en Facebook e Instagram a personas parecidas a tus mejores clientes.</t>
+          <t>Necesitamos tu ayuda con los datos de tus 20 clientes más leales (los que más te compran, los que renuevan sin problema).</t>
         </is>
       </c>
     </row>
@@ -581,14 +581,14 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Campos obligatorios: Nombre completo y Teléfono.</t>
+          <t>Campos obligatorios: Nombre completo, Teléfono y Email.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Campos opcionales (pero ayudan mucho a que el anuncio funcione mejor): Email, Ciudad, Estado, Código Postal, Género, Fecha de nacimiento o edad.</t>
+          <t>Campos opcionales (pero ayudan mucho): Ciudad, Estado, Código Postal, Género, Fecha de nacimiento o edad.</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Esta información es confidencial y solo se usa para publicidad en Facebook/Instagram. No se comparte con nadie más.</t>
+          <t>Esta información es confidencial y es solo para uso interno de Enlace Integral Seguros. No se comparte con nadie más.</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email *</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">

</xml_diff>